<commit_message>
Stat tests of HA assumptions
</commit_message>
<xml_diff>
--- a/Copper/6. Statistical data analysis/Plots by typology/Cu_species_relative_proportions.xlsx
+++ b/Copper/6. Statistical data analysis/Plots by typology/Cu_species_relative_proportions.xlsx
@@ -1,81 +1,70 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="29822"/>
-  <workbookPr/>
-  <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
-    <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://ornl-my.sharepoint.com/personal/q4q_ornl_gov/Documents/Research/Bioavailability Project/BLM_spatial_assessmt/Copper/6. Statistical data analysis/Plots by typology/"/>
-    </mc:Choice>
-  </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="19" documentId="11_C2CE303C78612A13875B34FC160A53129275A135" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{6D4BAADE-08A7-4C31-90D1-EE8F06AA1FAF}"/>
+  <workbookPr date1904="false"/>
   <bookViews>
-    <workbookView xWindow="-110" yWindow="-110" windowWidth="19420" windowHeight="11500" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="0" yWindow="0" windowWidth="13125" windowHeight="6105" firstSheet="0" activeTab="0"/>
   </bookViews>
   <sheets>
-    <sheet name="Sheet 1" sheetId="1" r:id="rId1"/>
+    <sheet name="Sheet 1" sheetId="1" state="visible" r:id="rId1"/>
   </sheets>
-  <calcPr calcId="0"/>
 </workbook>
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
 <sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="15" uniqueCount="15">
   <si>
-    <t>Typology</t>
-  </si>
-  <si>
-    <t>CuCO3_nM</t>
-  </si>
-  <si>
-    <t>CuCl_nM</t>
-  </si>
-  <si>
-    <t>CuHCO3_nM</t>
-  </si>
-  <si>
-    <t>CuOH_nM</t>
-  </si>
-  <si>
-    <t>CuSO4_nM</t>
-  </si>
-  <si>
-    <t>Cu_CO3_2_nM</t>
-  </si>
-  <si>
-    <t>Cu_OH_2_nM</t>
-  </si>
-  <si>
-    <t>Free_Cu_nM</t>
-  </si>
-  <si>
-    <t>TOrg_Cu_nM</t>
-  </si>
-  <si>
-    <t>Pooled</t>
-  </si>
-  <si>
-    <t>Non-Perennial</t>
-  </si>
-  <si>
-    <t>Perennial</t>
-  </si>
-  <si>
-    <t>Developed Perennial</t>
-  </si>
-  <si>
-    <t>Main Stem</t>
+    <t xml:space="preserve">Typology</t>
+  </si>
+  <si>
+    <t xml:space="preserve">CuCO3_nM</t>
+  </si>
+  <si>
+    <t xml:space="preserve">CuCl_nM</t>
+  </si>
+  <si>
+    <t xml:space="preserve">CuHCO3_nM</t>
+  </si>
+  <si>
+    <t xml:space="preserve">CuOH_nM</t>
+  </si>
+  <si>
+    <t xml:space="preserve">CuSO4_nM</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Cu_CO3_2_nM</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Cu_OH_2_nM</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Free_Cu_nM</t>
+  </si>
+  <si>
+    <t xml:space="preserve">TOrg_Cu_nM</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Pooled</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Non-Perennial</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Perennial</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Developed Perennial</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Main Stem</t>
   </si>
 </sst>
 </file>
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
-  <numFmts count="2">
-    <numFmt numFmtId="167" formatCode="0.000"/>
-    <numFmt numFmtId="170" formatCode="0.0"/>
-  </numFmts>
-  <fonts count="1" x14ac:knownFonts="1">
+  <numFmts count="0"/>
+  <fonts count="1">
     <font>
       <sz val="11"/>
       <color rgb="FF000000"/>
@@ -104,26 +93,13 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="5">
+  <cellXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
-    <xf numFmtId="167" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
-    <xf numFmtId="11" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
-    <xf numFmtId="2" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
-    <xf numFmtId="170" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
   </cellStyles>
   <dxfs count="0"/>
-  <tableStyles count="0" defaultTableStyle="TableStyleMedium2" defaultPivotStyle="PivotStyleLight16"/>
-  <extLst>
-    <ext xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" uri="{EB79DEF2-80B8-43e5-95BD-54CBDDF9020C}">
-      <x14:slicerStyles defaultSlicerStyle="SlicerStyleLight1"/>
-    </ext>
-    <ext xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" uri="{9260A510-F301-46a8-8635-F512D64BE5F5}">
-      <x15:timelineStyles defaultTimelineStyle="TimeSlicerStyleLight1"/>
-    </ext>
-  </extLst>
 </styleSheet>
 </file>
 
@@ -405,11 +381,11 @@
 </file>
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
-  <dimension ref="A1:J6"/>
-  <sheetFormatPr defaultColWidth="10.90625" defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3">
+  <dimension ref="A1"/>
+  <sheetFormatPr defaultRowHeight="15.0" baseColWidth="10"/>
   <sheetData>
-    <row r="1" spans="1:10" x14ac:dyDescent="0.35">
+    <row r="1">
       <c r="A1" t="s">
         <v>0</v>
       </c>
@@ -441,174 +417,168 @@
         <v>9</v>
       </c>
     </row>
-    <row r="2" spans="1:10" x14ac:dyDescent="0.35">
+    <row r="2">
       <c r="A2" t="s">
         <v>10</v>
       </c>
-      <c r="B2" s="1">
-        <v>0.81967826925258203</v>
-      </c>
-      <c r="C2" s="2">
-        <v>1.5034629001270299E-4</v>
-      </c>
-      <c r="D2" s="3">
-        <v>6.0903051817722504</v>
-      </c>
-      <c r="E2" s="2">
-        <v>2.1469502191875E-2</v>
-      </c>
-      <c r="F2" s="2">
-        <v>1.2377539368229301E-3</v>
-      </c>
-      <c r="G2" s="2">
-        <v>2.2928193325833001E-3</v>
-      </c>
-      <c r="H2" s="2">
-        <v>3.6355113453998803E-4</v>
-      </c>
-      <c r="I2" s="2">
-        <v>0.21012023331836899</v>
-      </c>
-      <c r="J2" s="4">
-        <v>92.854382342771004</v>
+      <c r="B2" t="n">
+        <v>0.819678269252582</v>
+      </c>
+      <c r="C2" t="n">
+        <v>0.000150346290012703</v>
+      </c>
+      <c r="D2" t="n">
+        <v>6.09030518177225</v>
+      </c>
+      <c r="E2" t="n">
+        <v>0.021469502191875</v>
+      </c>
+      <c r="F2" t="n">
+        <v>0.00123775393682293</v>
+      </c>
+      <c r="G2" t="n">
+        <v>0.0022928193325833</v>
+      </c>
+      <c r="H2" t="n">
+        <v>0.000363551134539988</v>
+      </c>
+      <c r="I2" t="n">
+        <v>0.210120233318369</v>
+      </c>
+      <c r="J2" t="n">
+        <v>92.854382342771</v>
       </c>
     </row>
-    <row r="3" spans="1:10" x14ac:dyDescent="0.35">
+    <row r="3">
       <c r="A3" t="s">
         <v>11</v>
       </c>
-      <c r="B3">
-        <v>0.13266494803524601</v>
-      </c>
-      <c r="C3">
-        <v>3.56989702717991E-5</v>
-      </c>
-      <c r="D3">
-        <v>0.50795737188353995</v>
-      </c>
-      <c r="E3">
-        <v>1.93249624835484E-2</v>
-      </c>
-      <c r="F3">
-        <v>1.250948260964E-3</v>
-      </c>
-      <c r="G3">
-        <v>2.6421496628805898E-4</v>
-      </c>
-      <c r="H3">
-        <v>9.8005828266133402E-4</v>
-      </c>
-      <c r="I3">
-        <v>0.17862877287541601</v>
-      </c>
-      <c r="J3">
-        <v>99.158893024242104</v>
+      <c r="B3" t="n">
+        <v>0.132664948035246</v>
+      </c>
+      <c r="C3" t="n">
+        <v>0.0000356989702717991</v>
+      </c>
+      <c r="D3" t="n">
+        <v>0.50795737188354</v>
+      </c>
+      <c r="E3" t="n">
+        <v>0.0193249624835484</v>
+      </c>
+      <c r="F3" t="n">
+        <v>0.001250948260964</v>
+      </c>
+      <c r="G3" t="n">
+        <v>0.000264214966288059</v>
+      </c>
+      <c r="H3" t="n">
+        <v>0.000980058282661334</v>
+      </c>
+      <c r="I3" t="n">
+        <v>0.178628772875416</v>
+      </c>
+      <c r="J3" t="n">
+        <v>99.1588930242421</v>
       </c>
     </row>
-    <row r="4" spans="1:10" x14ac:dyDescent="0.35">
+    <row r="4">
       <c r="A4" t="s">
         <v>12</v>
       </c>
-      <c r="B4">
-        <v>0.85564987164975304</v>
-      </c>
-      <c r="C4">
-        <v>1.43887990626775E-5</v>
-      </c>
-      <c r="D4">
+      <c r="B4" t="n">
+        <v>0.855649871649753</v>
+      </c>
+      <c r="C4" t="n">
+        <v>0.0000143887990626775</v>
+      </c>
+      <c r="D4" t="n">
         <v>1.67772602496403</v>
       </c>
-      <c r="E4">
-        <v>3.4738363959623798E-2</v>
-      </c>
-      <c r="F4">
-        <v>5.2942991958834405E-4</v>
-      </c>
-      <c r="G4">
-        <v>9.1593231992683002E-3</v>
-      </c>
-      <c r="H4">
-        <v>2.3253995685589999E-3</v>
-      </c>
-      <c r="I4">
-        <v>7.6527807883086593E-2</v>
-      </c>
-      <c r="J4">
-        <v>97.343329390056994</v>
+      <c r="E4" t="n">
+        <v>0.0347383639596238</v>
+      </c>
+      <c r="F4" t="n">
+        <v>0.000529429919588344</v>
+      </c>
+      <c r="G4" t="n">
+        <v>0.0091593231992683</v>
+      </c>
+      <c r="H4" t="n">
+        <v>0.002325399568559</v>
+      </c>
+      <c r="I4" t="n">
+        <v>0.0765278078830866</v>
+      </c>
+      <c r="J4" t="n">
+        <v>97.343329390057</v>
       </c>
     </row>
-    <row r="5" spans="1:10" x14ac:dyDescent="0.35">
+    <row r="5">
       <c r="A5" t="s">
         <v>13</v>
       </c>
-      <c r="B5">
+      <c r="B5" t="n">
         <v>3.1235359509856</v>
       </c>
-      <c r="C5">
-        <v>1.2001233485873499E-4</v>
-      </c>
-      <c r="D5">
-        <v>8.2612599161162592</v>
-      </c>
-      <c r="E5">
-        <v>8.7075770665403895E-2</v>
-      </c>
-      <c r="F5">
-        <v>1.28770437520152E-3</v>
-      </c>
-      <c r="G5">
-        <v>3.3360718316446603E-2</v>
-      </c>
-      <c r="H5">
-        <v>4.4725072977722597E-3</v>
-      </c>
-      <c r="I5">
-        <v>0.26654881289390098</v>
-      </c>
-      <c r="J5">
-        <v>88.222338607014606</v>
+      <c r="C5" t="n">
+        <v>0.000120012334858735</v>
+      </c>
+      <c r="D5" t="n">
+        <v>8.26125991611626</v>
+      </c>
+      <c r="E5" t="n">
+        <v>0.0870757706654039</v>
+      </c>
+      <c r="F5" t="n">
+        <v>0.00128770437520152</v>
+      </c>
+      <c r="G5" t="n">
+        <v>0.0333607183164466</v>
+      </c>
+      <c r="H5" t="n">
+        <v>0.00447250729777226</v>
+      </c>
+      <c r="I5" t="n">
+        <v>0.266548812893901</v>
+      </c>
+      <c r="J5" t="n">
+        <v>88.2223386070146</v>
       </c>
     </row>
-    <row r="6" spans="1:10" x14ac:dyDescent="0.35">
+    <row r="6">
       <c r="A6" t="s">
         <v>14</v>
       </c>
-      <c r="B6">
-        <v>1.5066188871558599</v>
-      </c>
-      <c r="C6">
-        <v>4.0438781955253398E-5</v>
-      </c>
-      <c r="D6">
-        <v>1.5537319600066599</v>
-      </c>
-      <c r="E6">
-        <v>4.4624762793555497E-2</v>
-      </c>
-      <c r="F6">
-        <v>1.0024218052356499E-3</v>
-      </c>
-      <c r="G6">
-        <v>5.31770960210027E-2</v>
-      </c>
-      <c r="H6">
-        <v>9.4241462743384404E-3</v>
-      </c>
-      <c r="I6">
-        <v>4.7744535243742003E-2</v>
-      </c>
-      <c r="J6">
+      <c r="B6" t="n">
+        <v>1.50661888715586</v>
+      </c>
+      <c r="C6" t="n">
+        <v>0.0000404387819552534</v>
+      </c>
+      <c r="D6" t="n">
+        <v>1.55373196000666</v>
+      </c>
+      <c r="E6" t="n">
+        <v>0.0446247627935555</v>
+      </c>
+      <c r="F6" t="n">
+        <v>0.00100242180523565</v>
+      </c>
+      <c r="G6" t="n">
+        <v>0.0531770960210027</v>
+      </c>
+      <c r="H6" t="n">
+        <v>0.00942414627433844</v>
+      </c>
+      <c r="I6" t="n">
+        <v>0.047744535243742</v>
+      </c>
+      <c r="J6" t="n">
         <v>96.7836357519177</v>
       </c>
     </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
-  <pageSetup paperSize="9" orientation="portrait" horizontalDpi="300" verticalDpi="300"/>
+  <pageSetup paperSize="9" orientation="portrait" horizontalDpi="300" verticalDpi="300" r:id="rId2"/>
 </worksheet>
-</file>
-
-<file path=docMetadata/LabelInfo.xml><?xml version="1.0" encoding="utf-8"?>
-<clbl:labelList xmlns:clbl="http://schemas.microsoft.com/office/2020/mipLabelMetadata">
-  <clbl:label id="{db3dbd43-4c4b-4544-9f8a-0553f9f5f25e}" enabled="0" method="" siteId="{db3dbd43-4c4b-4544-9f8a-0553f9f5f25e}" removed="1"/>
-</clbl:labelList>
 </file>
</xml_diff>